<commit_message>
client command table updated
</commit_message>
<xml_diff>
--- a/questions/Client Command Table A9.xlsx
+++ b/questions/Client Command Table A9.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nalin\SimplicityStudio\v5_workspace\ecen5823-assignment7-nasa7792\questions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nalin\SimplicityStudio\v5_workspace\ecen5823-assignment9-nasa7792\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55BC87E-7A5E-4ECA-97AF-F04C0FC7CB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{420755EF-44AC-4B64-A7B6-C807F34A183B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
-  <si>
-    <t>Client Command Table for A7</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
   <si>
     <t>Use this table to help you design your program. Add rows as needed.</t>
   </si>
@@ -88,27 +85,12 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Events Common to Slaves/Clients</t>
-  </si>
-  <si>
     <t>sl_bt_evt_system_boot_id</t>
   </si>
   <si>
     <t>This event is generated on stack boot up</t>
   </si>
   <si>
-    <t>sl_bt_scanner_set_mode()</t>
-  </si>
-  <si>
-    <t>sl_bt_scanner_set_timing()</t>
-  </si>
-  <si>
-    <t>sl_bt_connection_set_default_parameters()</t>
-  </si>
-  <si>
-    <t>sl_bt_scanner_start()</t>
-  </si>
-  <si>
     <t>sl_bt_evt_connection_opened_id</t>
   </si>
   <si>
@@ -118,57 +100,19 @@
     <t>sl_bt_evt_system_soft_timer_id</t>
   </si>
   <si>
-    <t>This event indicates that a soft timer has expired.</t>
-  </si>
-  <si>
-    <t>Events only for Masters/Clients</t>
-  </si>
-  <si>
     <t>sl_bt_evt_scanner_scan_report_id</t>
   </si>
   <si>
-    <t>Received for advertising or scan response packets generated by: sl_bt_scanner_start().
-Is the bd_addr, packet_type and address_type what we expect for our Server? If yes:
-   sl_bt_scanner_stop()
-   sl_bt_connection_open()</t>
-  </si>
-  <si>
     <t>sl_bt_evt_gatt_procedure_completed_id</t>
   </si>
   <si>
-    <t>We get this event when it’s ok to call the next GATT command. It’s a good idea to check for returned error codes. This would be a great event to use to sequence your new state machine.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do not build your state machine into your  handle_ble_event() function! Instead build a new state machine for A7. </t>
-  </si>
-  <si>
     <t>sl_bt_evt_gatt_service_id</t>
   </si>
   <si>
-    <t>A GATT service in the remote GATT database was discovered</t>
-  </si>
-  <si>
     <t>sl_bt_evt_gatt_characteristic_id</t>
   </si>
   <si>
-    <t>A GATT characteristic in the remote GATT database was discovered</t>
-  </si>
-  <si>
     <t>sl_bt_evt_gatt_characteristic_value_id</t>
-  </si>
-  <si>
-    <t>If an indication or notification has been enabled for a characteristic, this event is triggered whenever an indication or notification is received from the remote GATT server.
-Is the characteristic handle and att_opcode we expect? If yes: 
-   sl_bt_gatt_send_characteristic_confirmation()</t>
-  </si>
-  <si>
-    <t>displayUpdate() to periodically refresh the lcd screen.</t>
-  </si>
-  <si>
-    <t>sl_bt_system_get_identity_address()
-sl_bt_advertiser_create_set()
-sl_bt_advertiser_set_timing()
-sl_bt_advertiser_start()</t>
   </si>
   <si>
     <t>sl_bt_advertiser_stop()
@@ -178,100 +122,11 @@
     <t>sl_bt_advertiser_start()</t>
   </si>
   <si>
-    <t xml:space="preserve">
-On boot up of the ble stack we need to call 4 events
-sl_bt_system_get_identity_address- helps fetch an address for the BLE device
-sl_bt_advertiser_create_set()-creats an advertising set
-sl_bt_advertiser_set_timing()- configures parameters related to advertising
-sl_bt_advertiser_start()- starts the advertising process and mark device as scannable
-</t>
-  </si>
-  <si>
     <t>once an active connection is in place we need to stop advertising by calling sl_bt_advertiser_stop()
 sl_bt_connection_set_parameters()-to change connection parameters of a Bluetooth connection.</t>
   </si>
   <si>
-    <t>on connection close, we start advertising again</t>
-  </si>
-  <si>
     <t>we call this update function to periodically refresh lcd to prevent damage.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>DISPLAY_ROW_NAME</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">- either displays client or server depending on device
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>DISPLAY_ROW_BTADDR-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> displays either the client's or server's address
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>DISPLAY_ROW_ASSIGNMEN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">T- shows A7
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>DISPLAY_ROW_CONNECTION</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>- for client- discovering for server advertising</t>
-    </r>
   </si>
   <si>
     <t>sl_bt_scanner_stop()
@@ -279,25 +134,7 @@
 no change to discovery state machine</t>
   </si>
   <si>
-    <t>base on current state the state changes 
-if we are in DISCOVER_SERVICES we move to DISCOVER_CHARACTERISTICS
-if we are in DISCOVER_CHARACTERISTICS we move to ENABLE_INDICATIONS
-if we are in STATE3_ENABLE_INDICATIONS we can move back to idle</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> no change to state , we store service handle</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> no change to state we store characterstic handle</t>
-  </si>
-  <si>
-    <t>no change to state , we send confirmation for indications and display the temperature on screen</t>
-  </si>
-  <si>
     <t>Not applicable</t>
-  </si>
-  <si>
-    <t>for client we also display the connected server's address in the row DISPLAY_ROW_BTADDR2</t>
   </si>
   <si>
     <r>
@@ -329,6 +166,78 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Refresh lcd with new temperature data for client in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISPLAY_ROW_TEMPVALUE</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISPLAY_ROW_NAME</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">- Client
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISPLAY_ROW_BTADDR-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> displays either the client's address
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISPLAY_ROW_ASSIGNMEN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">T- shows A9
+</t>
+    </r>
+    <r>
       <rPr>
         <b/>
         <sz val="10"/>
@@ -343,15 +252,30 @@
         <sz val="10"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> client" displays discovering 
-master displays advertising</t>
+      <t>- for discovering</t>
     </r>
   </si>
   <si>
+    <t xml:space="preserve">
+sl_bt_system_get_identity_address- helps fetch an address for the BLE device
+sl_bt_advertiser_create_set()-creats an advertising set
+sl_bt_advertiser_set_timing()- configures parameters related to advertising
+sl_bt_advertiser_start()- starts the advertising process and mark device as scannable
+from A9
+we also need to call sl_bt_sm_delete_bondings() to clear any previous bondings and sl_bt_sm_configure to add security in the form of yes no during bonding</t>
+  </si>
+  <si>
+    <t>sl_bt_sm_delete_bondings()- we need to clear all previous bondings
+sl_bt_sm_configure()- security apis
+sl_bt_system_get_identity_address()
+sl_bt_advertiser_create_set()
+sl_bt_advertiser_set_timing()
+sl_bt_advertiser_start()</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">Refresh lcd with new temperature data for client in the </t>
+      <t xml:space="preserve">for client we display the connected server's address in the row </t>
     </r>
     <r>
       <rPr>
@@ -361,15 +285,102 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>DISPLAY_ROW_TEMPVALUE</t>
+      <t>DISPLAY_ROW_BTADDR2</t>
     </r>
+  </si>
+  <si>
+    <t>Yes the event causes a state change</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>DISPLAY_ROW_CONNECTION-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">discovering 
+</t>
+    </r>
+  </si>
+  <si>
+    <t>on connection close, we start advertising again, we need to be careful here and do a proper cleanup and call sl_bt_sm_delete_bondings() and reset all the flags used to their default values</t>
+  </si>
+  <si>
+    <t>No change to state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client events </t>
+  </si>
+  <si>
+    <t>No change to state machine</t>
+  </si>
+  <si>
+    <t>we found an advertising packet from a known server, we open a new connection and stop scanning</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no change to state , we store service handle of both button and htm services</t>
+  </si>
+  <si>
+    <t>base on current state the state changes 
+if we are in STATE1_DISCOVER_HTM_SERVICE we move to STATE2_DISCOVER_HTM_CHARACTERISTICS
+if we are in STATE2_DISCOVER_HTM_CHARACTERISTICS we move to STATE3_ENABLE_HTM_INDICATIONS
+if we are in STATE3_ENABLE_HTM_INDICATIONS S we can move back to STATE4_DISCOVER_BTN_SERVICE,
+STATE4_DISCOVER_BTN_SERVICE,-&gt; STATE5_DISCOVER_BTN_CHARACTERISTICS
+ STATE5_DISCOVER_BTN_CHARACTERISTICS-&gt;STATE6_ENABLE_BTN_INDICATIONS
+STATE6_ENABLE_BTN_INDICATIONS-&gt;STATE0_IDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no change to state we store characterstic handle of htm and button service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no change to state </t>
+  </si>
+  <si>
+    <t>, we send confirmation for indications and display the temperature on screen, we also display changes to button service if indications are enabled</t>
+  </si>
+  <si>
+    <t>sl_bt_gatt_send_characteristic_confirmation()</t>
+  </si>
+  <si>
+    <t>no change to state</t>
+  </si>
+  <si>
+    <t>The first time we press PB1 , we get an error to raise security this triggers the bonding step</t>
+  </si>
+  <si>
+    <t>sl_bt_sm_increase_security</t>
+  </si>
+  <si>
+    <t>Client Command Table for A9</t>
+  </si>
+  <si>
+    <t>sl_bt_evt_system_external_signal_id</t>
+  </si>
+  <si>
+    <t>toggles the button indication for a special sequence of PB0 and PB1
+The first press of PB1 triggers bonding</t>
+  </si>
+  <si>
+    <t>sl_bt_gatt_set_characteristic_notification
+sl_bt_gatt_read_characteristic_value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -433,6 +444,23 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -448,7 +476,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -538,11 +566,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -597,16 +664,39 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1770,12 +1860,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="35" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="39.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="44" style="1" customWidth="1"/>
     <col min="5" max="5" width="49.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="44.88671875" style="1" customWidth="1"/>
@@ -1785,8 +1875,8 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="22" t="s">
-        <v>0</v>
+      <c r="B1" s="33" t="s">
+        <v>48</v>
       </c>
       <c r="C1" s="23"/>
       <c r="D1" s="23"/>
@@ -1804,40 +1894,40 @@
     <row r="3" spans="1:6" ht="119.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>3</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>4</v>
       </c>
       <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="5" spans="1:6" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>10</v>
+      <c r="A5" s="27" t="s">
+        <v>36</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="9"/>
@@ -1850,35 +1940,33 @@
       <c r="C6" s="9"/>
       <c r="D6" s="10"/>
       <c r="E6" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" ht="221.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>37</v>
+        <v>32</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="13"/>
-      <c r="E8" s="14" t="s">
-        <v>14</v>
-      </c>
+      <c r="E8" s="14"/>
       <c r="F8" s="15"/>
     </row>
     <row r="9" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1886,9 +1974,7 @@
       <c r="B9" s="4"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="14" t="s">
-        <v>15</v>
-      </c>
+      <c r="E9" s="26"/>
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" ht="26.7" customHeight="1" x14ac:dyDescent="0.3">
@@ -1896,9 +1982,7 @@
       <c r="B10" s="4"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="14" t="s">
-        <v>16</v>
-      </c>
+      <c r="E10" s="14"/>
       <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1912,17 +1996,19 @@
     <row r="12" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="17" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="D12" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="16"/>
+      <c r="E12" s="20" t="s">
+        <v>19</v>
+      </c>
       <c r="F12" s="16" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1936,17 +2022,19 @@
     <row r="14" spans="1:6" ht="154.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="17" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16" t="s">
-        <v>39</v>
+        <v>35</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1960,19 +2048,17 @@
     <row r="16" spans="1:6" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>20</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E16" s="18"/>
       <c r="F16" s="16" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1984,9 +2070,7 @@
       <c r="F17" s="16"/>
     </row>
     <row r="18" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>21</v>
-      </c>
+      <c r="A18" s="7"/>
       <c r="B18" s="4"/>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
@@ -1995,19 +2079,21 @@
     </row>
     <row r="19" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
-      <c r="B19" s="25" t="s">
-        <v>22</v>
+      <c r="B19" s="22" t="s">
+        <v>14</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="E19" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="16"/>
+      <c r="F19" s="20" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
@@ -2017,23 +2103,19 @@
       <c r="E20" s="19"/>
       <c r="F20" s="16"/>
     </row>
-    <row r="21" spans="1:6" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="239.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="17" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="E21" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>26</v>
-      </c>
+      <c r="D21" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="18"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
@@ -2043,20 +2125,18 @@
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="17" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>28</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="18"/>
       <c r="F23" s="16"/>
     </row>
     <row r="24" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2070,17 +2150,15 @@
     <row r="25" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="17" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>30</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" s="18"/>
       <c r="F25" s="16"/>
     </row>
     <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2093,19 +2171,21 @@
     </row>
     <row r="27" spans="1:6" ht="65.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
-      <c r="B27" s="17" t="s">
-        <v>31</v>
+      <c r="B27" s="22" t="s">
+        <v>18</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="F27" s="16"/>
+        <v>27</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
@@ -2117,11 +2197,51 @@
     </row>
     <row r="29" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="B29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="31"/>
+      <c r="B30" s="4"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+    </row>
+    <row r="31" spans="1:6" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C32" s="30"/>
+    </row>
+    <row r="33" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>